<commit_message>
Recimo da zaključen app
</commit_message>
<xml_diff>
--- a/SP 2026 - tekme.xlsx
+++ b/SP 2026 - tekme.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="8985" yWindow="5115" windowWidth="28800" windowHeight="15345" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="150" yWindow="150" windowWidth="23010" windowHeight="13650" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tekme" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Skupine" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Tekme" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Skupine" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" calcMode="manual" fullCalcOnLoad="1"/>
@@ -838,7 +838,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1201,7 +1201,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>D</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -3052,7 +3052,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>D</t>
         </is>
       </c>
     </row>

</xml_diff>